<commit_message>
Small change to week 11 example
</commit_message>
<xml_diff>
--- a/Module 3/Week 11 - Short sales and dollar-neutral strategies/Example with value and growth stocks.xlsx
+++ b/Module 3/Week 11 - Short sales and dollar-neutral strategies/Example with value and growth stocks.xlsx
@@ -8,9 +8,9 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Analysis" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="At 1% exc return vol" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="Data" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Analysis" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="At 1% exc return vol" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -39,13 +39,13 @@
     <t xml:space="preserve">Growth</t>
   </si>
   <si>
-    <t xml:space="preserve">Market exc</t>
+    <t xml:space="preserve">Market excess</t>
   </si>
   <si>
-    <t xml:space="preserve">Value exc</t>
+    <t xml:space="preserve">Value excess</t>
   </si>
   <si>
-    <t xml:space="preserve">Growth exc</t>
+    <t xml:space="preserve">Growth excess</t>
   </si>
   <si>
     <t xml:space="preserve">Value minus growth</t>
@@ -161,7 +161,7 @@
     <numFmt numFmtId="167" formatCode="0.0000"/>
     <numFmt numFmtId="168" formatCode="[$$-409]#,##0.00;[RED]\-[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -191,12 +191,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u val="single"/>
@@ -256,44 +250,48 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -309,8 +307,114 @@
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+  <a:themeElements>
+    <a:clrScheme name="LibreOffice">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="ffffff"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="000000"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="ffffff"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="18a303"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="0369a3"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="a33e03"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8e03a3"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="c99c00"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="c9211e"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000ee"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="551a8b"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
+        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme>
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:prstDash val="solid"/>
+          <a:miter/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -318,43 +422,43 @@
   <sheetFormatPr defaultColWidth="8.6953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="8.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="18.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="10.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="9.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="18.24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="K1" s="0" t="s">
+      <c r="K1" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="n">
+      <c r="A2" s="5" t="n">
         <v>25934</v>
       </c>
       <c r="B2" s="1" t="n">
@@ -387,7 +491,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="5" t="n">
         <v>25965</v>
       </c>
       <c r="B3" s="1" t="n">
@@ -420,7 +524,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="5" t="n">
         <v>25993</v>
       </c>
       <c r="B4" s="1" t="n">
@@ -453,7 +557,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>26024</v>
       </c>
       <c r="B5" s="1" t="n">
@@ -486,7 +590,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>26054</v>
       </c>
       <c r="B6" s="1" t="n">
@@ -519,7 +623,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>26085</v>
       </c>
       <c r="B7" s="1" t="n">
@@ -552,7 +656,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="A8" s="5" t="n">
         <v>26115</v>
       </c>
       <c r="B8" s="1" t="n">
@@ -585,7 +689,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>26146</v>
       </c>
       <c r="B9" s="1" t="n">
@@ -618,7 +722,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="5" t="n">
         <v>26177</v>
       </c>
       <c r="B10" s="1" t="n">
@@ -651,7 +755,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
+      <c r="A11" s="5" t="n">
         <v>26207</v>
       </c>
       <c r="B11" s="1" t="n">
@@ -684,7 +788,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
+      <c r="A12" s="5" t="n">
         <v>26238</v>
       </c>
       <c r="B12" s="1" t="n">
@@ -717,7 +821,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
+      <c r="A13" s="5" t="n">
         <v>26268</v>
       </c>
       <c r="B13" s="1" t="n">
@@ -750,7 +854,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
+      <c r="A14" s="5" t="n">
         <v>26299</v>
       </c>
       <c r="B14" s="1" t="n">
@@ -783,7 +887,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
+      <c r="A15" s="5" t="n">
         <v>26330</v>
       </c>
       <c r="B15" s="1" t="n">
@@ -816,7 +920,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
+      <c r="A16" s="5" t="n">
         <v>26359</v>
       </c>
       <c r="B16" s="1" t="n">
@@ -849,7 +953,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
+      <c r="A17" s="5" t="n">
         <v>26390</v>
       </c>
       <c r="B17" s="1" t="n">
@@ -882,7 +986,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
+      <c r="A18" s="5" t="n">
         <v>26420</v>
       </c>
       <c r="B18" s="1" t="n">
@@ -915,7 +1019,7 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="5" t="n">
         <v>26451</v>
       </c>
       <c r="B19" s="1" t="n">
@@ -948,7 +1052,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
+      <c r="A20" s="5" t="n">
         <v>26481</v>
       </c>
       <c r="B20" s="1" t="n">
@@ -981,7 +1085,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="5" t="n">
         <v>26512</v>
       </c>
       <c r="B21" s="1" t="n">
@@ -1014,7 +1118,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
+      <c r="A22" s="5" t="n">
         <v>26543</v>
       </c>
       <c r="B22" s="1" t="n">
@@ -1047,7 +1151,7 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
+      <c r="A23" s="5" t="n">
         <v>26573</v>
       </c>
       <c r="B23" s="1" t="n">
@@ -1080,7 +1184,7 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
+      <c r="A24" s="5" t="n">
         <v>26604</v>
       </c>
       <c r="B24" s="1" t="n">
@@ -1113,7 +1217,7 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
+      <c r="A25" s="5" t="n">
         <v>26634</v>
       </c>
       <c r="B25" s="1" t="n">
@@ -1146,7 +1250,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
+      <c r="A26" s="5" t="n">
         <v>26665</v>
       </c>
       <c r="B26" s="1" t="n">
@@ -1179,7 +1283,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
+      <c r="A27" s="5" t="n">
         <v>26696</v>
       </c>
       <c r="B27" s="1" t="n">
@@ -1212,7 +1316,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="n">
+      <c r="A28" s="5" t="n">
         <v>26724</v>
       </c>
       <c r="B28" s="1" t="n">
@@ -1245,7 +1349,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="n">
+      <c r="A29" s="5" t="n">
         <v>26755</v>
       </c>
       <c r="B29" s="1" t="n">
@@ -1278,7 +1382,7 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="n">
+      <c r="A30" s="5" t="n">
         <v>26785</v>
       </c>
       <c r="B30" s="1" t="n">
@@ -1311,7 +1415,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="n">
+      <c r="A31" s="5" t="n">
         <v>26816</v>
       </c>
       <c r="B31" s="1" t="n">
@@ -1344,7 +1448,7 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="n">
+      <c r="A32" s="5" t="n">
         <v>26846</v>
       </c>
       <c r="B32" s="1" t="n">
@@ -1377,7 +1481,7 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="n">
+      <c r="A33" s="5" t="n">
         <v>26877</v>
       </c>
       <c r="B33" s="1" t="n">
@@ -1410,7 +1514,7 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="n">
+      <c r="A34" s="5" t="n">
         <v>26908</v>
       </c>
       <c r="B34" s="1" t="n">
@@ -1443,7 +1547,7 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="n">
+      <c r="A35" s="5" t="n">
         <v>26938</v>
       </c>
       <c r="B35" s="1" t="n">
@@ -1476,7 +1580,7 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="n">
+      <c r="A36" s="5" t="n">
         <v>26969</v>
       </c>
       <c r="B36" s="1" t="n">
@@ -1509,7 +1613,7 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="n">
+      <c r="A37" s="5" t="n">
         <v>26999</v>
       </c>
       <c r="B37" s="1" t="n">
@@ -1542,7 +1646,7 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="n">
+      <c r="A38" s="5" t="n">
         <v>27030</v>
       </c>
       <c r="B38" s="1" t="n">
@@ -1575,7 +1679,7 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="n">
+      <c r="A39" s="5" t="n">
         <v>27061</v>
       </c>
       <c r="B39" s="1" t="n">
@@ -1608,7 +1712,7 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="n">
+      <c r="A40" s="5" t="n">
         <v>27089</v>
       </c>
       <c r="B40" s="1" t="n">
@@ -1641,7 +1745,7 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="n">
+      <c r="A41" s="5" t="n">
         <v>27120</v>
       </c>
       <c r="B41" s="1" t="n">
@@ -1674,7 +1778,7 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="n">
+      <c r="A42" s="5" t="n">
         <v>27150</v>
       </c>
       <c r="B42" s="1" t="n">
@@ -1707,7 +1811,7 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="n">
+      <c r="A43" s="5" t="n">
         <v>27181</v>
       </c>
       <c r="B43" s="1" t="n">
@@ -1740,7 +1844,7 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="n">
+      <c r="A44" s="5" t="n">
         <v>27211</v>
       </c>
       <c r="B44" s="1" t="n">
@@ -1773,7 +1877,7 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="n">
+      <c r="A45" s="5" t="n">
         <v>27242</v>
       </c>
       <c r="B45" s="1" t="n">
@@ -1806,7 +1910,7 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="n">
+      <c r="A46" s="5" t="n">
         <v>27273</v>
       </c>
       <c r="B46" s="1" t="n">
@@ -1839,7 +1943,7 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="n">
+      <c r="A47" s="5" t="n">
         <v>27303</v>
       </c>
       <c r="B47" s="1" t="n">
@@ -1872,7 +1976,7 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="n">
+      <c r="A48" s="5" t="n">
         <v>27334</v>
       </c>
       <c r="B48" s="1" t="n">
@@ -1905,7 +2009,7 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="n">
+      <c r="A49" s="5" t="n">
         <v>27364</v>
       </c>
       <c r="B49" s="1" t="n">
@@ -1938,7 +2042,7 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="n">
+      <c r="A50" s="5" t="n">
         <v>27395</v>
       </c>
       <c r="B50" s="1" t="n">
@@ -1971,7 +2075,7 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="n">
+      <c r="A51" s="5" t="n">
         <v>27426</v>
       </c>
       <c r="B51" s="1" t="n">
@@ -2004,7 +2108,7 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="n">
+      <c r="A52" s="5" t="n">
         <v>27454</v>
       </c>
       <c r="B52" s="1" t="n">
@@ -2037,7 +2141,7 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="n">
+      <c r="A53" s="5" t="n">
         <v>27485</v>
       </c>
       <c r="B53" s="1" t="n">
@@ -2070,7 +2174,7 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="n">
+      <c r="A54" s="5" t="n">
         <v>27515</v>
       </c>
       <c r="B54" s="1" t="n">
@@ -2103,7 +2207,7 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="n">
+      <c r="A55" s="5" t="n">
         <v>27546</v>
       </c>
       <c r="B55" s="1" t="n">
@@ -2136,7 +2240,7 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="n">
+      <c r="A56" s="5" t="n">
         <v>27576</v>
       </c>
       <c r="B56" s="1" t="n">
@@ -2169,7 +2273,7 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="n">
+      <c r="A57" s="5" t="n">
         <v>27607</v>
       </c>
       <c r="B57" s="1" t="n">
@@ -2202,7 +2306,7 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4" t="n">
+      <c r="A58" s="5" t="n">
         <v>27638</v>
       </c>
       <c r="B58" s="1" t="n">
@@ -2235,7 +2339,7 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="n">
+      <c r="A59" s="5" t="n">
         <v>27668</v>
       </c>
       <c r="B59" s="1" t="n">
@@ -2268,7 +2372,7 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="4" t="n">
+      <c r="A60" s="5" t="n">
         <v>27699</v>
       </c>
       <c r="B60" s="1" t="n">
@@ -2301,7 +2405,7 @@
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="4" t="n">
+      <c r="A61" s="5" t="n">
         <v>27729</v>
       </c>
       <c r="B61" s="1" t="n">
@@ -2334,7 +2438,7 @@
       </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="4" t="n">
+      <c r="A62" s="5" t="n">
         <v>27760</v>
       </c>
       <c r="B62" s="1" t="n">
@@ -2367,7 +2471,7 @@
       </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="n">
+      <c r="A63" s="5" t="n">
         <v>27791</v>
       </c>
       <c r="B63" s="1" t="n">
@@ -2400,7 +2504,7 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="4" t="n">
+      <c r="A64" s="5" t="n">
         <v>27820</v>
       </c>
       <c r="B64" s="1" t="n">
@@ -2433,7 +2537,7 @@
       </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="4" t="n">
+      <c r="A65" s="5" t="n">
         <v>27851</v>
       </c>
       <c r="B65" s="1" t="n">
@@ -2466,7 +2570,7 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="4" t="n">
+      <c r="A66" s="5" t="n">
         <v>27881</v>
       </c>
       <c r="B66" s="1" t="n">
@@ -2499,7 +2603,7 @@
       </c>
     </row>
     <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="4" t="n">
+      <c r="A67" s="5" t="n">
         <v>27912</v>
       </c>
       <c r="B67" s="1" t="n">
@@ -2532,7 +2636,7 @@
       </c>
     </row>
     <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="4" t="n">
+      <c r="A68" s="5" t="n">
         <v>27942</v>
       </c>
       <c r="B68" s="1" t="n">
@@ -2565,7 +2669,7 @@
       </c>
     </row>
     <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="4" t="n">
+      <c r="A69" s="5" t="n">
         <v>27973</v>
       </c>
       <c r="B69" s="1" t="n">
@@ -2598,7 +2702,7 @@
       </c>
     </row>
     <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="4" t="n">
+      <c r="A70" s="5" t="n">
         <v>28004</v>
       </c>
       <c r="B70" s="1" t="n">
@@ -2631,7 +2735,7 @@
       </c>
     </row>
     <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="n">
+      <c r="A71" s="5" t="n">
         <v>28034</v>
       </c>
       <c r="B71" s="1" t="n">
@@ -2664,7 +2768,7 @@
       </c>
     </row>
     <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="n">
+      <c r="A72" s="5" t="n">
         <v>28065</v>
       </c>
       <c r="B72" s="1" t="n">
@@ -2697,7 +2801,7 @@
       </c>
     </row>
     <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A73" s="4" t="n">
+      <c r="A73" s="5" t="n">
         <v>28095</v>
       </c>
       <c r="B73" s="1" t="n">
@@ -2730,7 +2834,7 @@
       </c>
     </row>
     <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="4" t="n">
+      <c r="A74" s="5" t="n">
         <v>28126</v>
       </c>
       <c r="B74" s="1" t="n">
@@ -2763,7 +2867,7 @@
       </c>
     </row>
     <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="4" t="n">
+      <c r="A75" s="5" t="n">
         <v>28157</v>
       </c>
       <c r="B75" s="1" t="n">
@@ -2796,7 +2900,7 @@
       </c>
     </row>
     <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="4" t="n">
+      <c r="A76" s="5" t="n">
         <v>28185</v>
       </c>
       <c r="B76" s="1" t="n">
@@ -2829,7 +2933,7 @@
       </c>
     </row>
     <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="4" t="n">
+      <c r="A77" s="5" t="n">
         <v>28216</v>
       </c>
       <c r="B77" s="1" t="n">
@@ -2862,7 +2966,7 @@
       </c>
     </row>
     <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="4" t="n">
+      <c r="A78" s="5" t="n">
         <v>28246</v>
       </c>
       <c r="B78" s="1" t="n">
@@ -2895,7 +2999,7 @@
       </c>
     </row>
     <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="n">
+      <c r="A79" s="5" t="n">
         <v>28277</v>
       </c>
       <c r="B79" s="1" t="n">
@@ -2928,7 +3032,7 @@
       </c>
     </row>
     <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="4" t="n">
+      <c r="A80" s="5" t="n">
         <v>28307</v>
       </c>
       <c r="B80" s="1" t="n">
@@ -2961,7 +3065,7 @@
       </c>
     </row>
     <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="4" t="n">
+      <c r="A81" s="5" t="n">
         <v>28338</v>
       </c>
       <c r="B81" s="1" t="n">
@@ -2994,7 +3098,7 @@
       </c>
     </row>
     <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="4" t="n">
+      <c r="A82" s="5" t="n">
         <v>28369</v>
       </c>
       <c r="B82" s="1" t="n">
@@ -3027,7 +3131,7 @@
       </c>
     </row>
     <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="4" t="n">
+      <c r="A83" s="5" t="n">
         <v>28399</v>
       </c>
       <c r="B83" s="1" t="n">
@@ -3060,7 +3164,7 @@
       </c>
     </row>
     <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="4" t="n">
+      <c r="A84" s="5" t="n">
         <v>28430</v>
       </c>
       <c r="B84" s="1" t="n">
@@ -3093,7 +3197,7 @@
       </c>
     </row>
     <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="4" t="n">
+      <c r="A85" s="5" t="n">
         <v>28460</v>
       </c>
       <c r="B85" s="1" t="n">
@@ -3126,7 +3230,7 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="4" t="n">
+      <c r="A86" s="5" t="n">
         <v>28491</v>
       </c>
       <c r="B86" s="1" t="n">
@@ -3159,7 +3263,7 @@
       </c>
     </row>
     <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="4" t="n">
+      <c r="A87" s="5" t="n">
         <v>28522</v>
       </c>
       <c r="B87" s="1" t="n">
@@ -3192,7 +3296,7 @@
       </c>
     </row>
     <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="4" t="n">
+      <c r="A88" s="5" t="n">
         <v>28550</v>
       </c>
       <c r="B88" s="1" t="n">
@@ -3225,7 +3329,7 @@
       </c>
     </row>
     <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="4" t="n">
+      <c r="A89" s="5" t="n">
         <v>28581</v>
       </c>
       <c r="B89" s="1" t="n">
@@ -3258,7 +3362,7 @@
       </c>
     </row>
     <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="n">
+      <c r="A90" s="5" t="n">
         <v>28611</v>
       </c>
       <c r="B90" s="1" t="n">
@@ -3291,7 +3395,7 @@
       </c>
     </row>
     <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="4" t="n">
+      <c r="A91" s="5" t="n">
         <v>28642</v>
       </c>
       <c r="B91" s="1" t="n">
@@ -3324,7 +3428,7 @@
       </c>
     </row>
     <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A92" s="4" t="n">
+      <c r="A92" s="5" t="n">
         <v>28672</v>
       </c>
       <c r="B92" s="1" t="n">
@@ -3357,7 +3461,7 @@
       </c>
     </row>
     <row r="93" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="4" t="n">
+      <c r="A93" s="5" t="n">
         <v>28703</v>
       </c>
       <c r="B93" s="1" t="n">
@@ -3390,7 +3494,7 @@
       </c>
     </row>
     <row r="94" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="4" t="n">
+      <c r="A94" s="5" t="n">
         <v>28734</v>
       </c>
       <c r="B94" s="1" t="n">
@@ -3423,7 +3527,7 @@
       </c>
     </row>
     <row r="95" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A95" s="4" t="n">
+      <c r="A95" s="5" t="n">
         <v>28764</v>
       </c>
       <c r="B95" s="1" t="n">
@@ -3456,7 +3560,7 @@
       </c>
     </row>
     <row r="96" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A96" s="4" t="n">
+      <c r="A96" s="5" t="n">
         <v>28795</v>
       </c>
       <c r="B96" s="1" t="n">
@@ -3489,7 +3593,7 @@
       </c>
     </row>
     <row r="97" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A97" s="4" t="n">
+      <c r="A97" s="5" t="n">
         <v>28825</v>
       </c>
       <c r="B97" s="1" t="n">
@@ -3522,7 +3626,7 @@
       </c>
     </row>
     <row r="98" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="4" t="n">
+      <c r="A98" s="5" t="n">
         <v>28856</v>
       </c>
       <c r="B98" s="1" t="n">
@@ -3555,7 +3659,7 @@
       </c>
     </row>
     <row r="99" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A99" s="4" t="n">
+      <c r="A99" s="5" t="n">
         <v>28887</v>
       </c>
       <c r="B99" s="1" t="n">
@@ -3588,7 +3692,7 @@
       </c>
     </row>
     <row r="100" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="4" t="n">
+      <c r="A100" s="5" t="n">
         <v>28915</v>
       </c>
       <c r="B100" s="1" t="n">
@@ -3621,7 +3725,7 @@
       </c>
     </row>
     <row r="101" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A101" s="4" t="n">
+      <c r="A101" s="5" t="n">
         <v>28946</v>
       </c>
       <c r="B101" s="1" t="n">
@@ -3654,7 +3758,7 @@
       </c>
     </row>
     <row r="102" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A102" s="4" t="n">
+      <c r="A102" s="5" t="n">
         <v>28976</v>
       </c>
       <c r="B102" s="1" t="n">
@@ -3687,7 +3791,7 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="4" t="n">
+      <c r="A103" s="5" t="n">
         <v>29007</v>
       </c>
       <c r="B103" s="1" t="n">
@@ -3720,7 +3824,7 @@
       </c>
     </row>
     <row r="104" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A104" s="4" t="n">
+      <c r="A104" s="5" t="n">
         <v>29037</v>
       </c>
       <c r="B104" s="1" t="n">
@@ -3753,7 +3857,7 @@
       </c>
     </row>
     <row r="105" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A105" s="4" t="n">
+      <c r="A105" s="5" t="n">
         <v>29068</v>
       </c>
       <c r="B105" s="1" t="n">
@@ -3786,7 +3890,7 @@
       </c>
     </row>
     <row r="106" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A106" s="4" t="n">
+      <c r="A106" s="5" t="n">
         <v>29099</v>
       </c>
       <c r="B106" s="1" t="n">
@@ -3819,7 +3923,7 @@
       </c>
     </row>
     <row r="107" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A107" s="4" t="n">
+      <c r="A107" s="5" t="n">
         <v>29129</v>
       </c>
       <c r="B107" s="1" t="n">
@@ -3852,7 +3956,7 @@
       </c>
     </row>
     <row r="108" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A108" s="4" t="n">
+      <c r="A108" s="5" t="n">
         <v>29160</v>
       </c>
       <c r="B108" s="1" t="n">
@@ -3885,7 +3989,7 @@
       </c>
     </row>
     <row r="109" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A109" s="4" t="n">
+      <c r="A109" s="5" t="n">
         <v>29190</v>
       </c>
       <c r="B109" s="1" t="n">
@@ -3918,7 +4022,7 @@
       </c>
     </row>
     <row r="110" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A110" s="4" t="n">
+      <c r="A110" s="5" t="n">
         <v>29221</v>
       </c>
       <c r="B110" s="1" t="n">
@@ -3951,7 +4055,7 @@
       </c>
     </row>
     <row r="111" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A111" s="4" t="n">
+      <c r="A111" s="5" t="n">
         <v>29252</v>
       </c>
       <c r="B111" s="1" t="n">
@@ -3984,7 +4088,7 @@
       </c>
     </row>
     <row r="112" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A112" s="4" t="n">
+      <c r="A112" s="5" t="n">
         <v>29281</v>
       </c>
       <c r="B112" s="1" t="n">
@@ -4017,7 +4121,7 @@
       </c>
     </row>
     <row r="113" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A113" s="4" t="n">
+      <c r="A113" s="5" t="n">
         <v>29312</v>
       </c>
       <c r="B113" s="1" t="n">
@@ -4050,7 +4154,7 @@
       </c>
     </row>
     <row r="114" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A114" s="4" t="n">
+      <c r="A114" s="5" t="n">
         <v>29342</v>
       </c>
       <c r="B114" s="1" t="n">
@@ -4083,7 +4187,7 @@
       </c>
     </row>
     <row r="115" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A115" s="4" t="n">
+      <c r="A115" s="5" t="n">
         <v>29373</v>
       </c>
       <c r="B115" s="1" t="n">
@@ -4116,7 +4220,7 @@
       </c>
     </row>
     <row r="116" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A116" s="4" t="n">
+      <c r="A116" s="5" t="n">
         <v>29403</v>
       </c>
       <c r="B116" s="1" t="n">
@@ -4149,7 +4253,7 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="4" t="n">
+      <c r="A117" s="5" t="n">
         <v>29434</v>
       </c>
       <c r="B117" s="1" t="n">
@@ -4182,7 +4286,7 @@
       </c>
     </row>
     <row r="118" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A118" s="4" t="n">
+      <c r="A118" s="5" t="n">
         <v>29465</v>
       </c>
       <c r="B118" s="1" t="n">
@@ -4215,7 +4319,7 @@
       </c>
     </row>
     <row r="119" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A119" s="4" t="n">
+      <c r="A119" s="5" t="n">
         <v>29495</v>
       </c>
       <c r="B119" s="1" t="n">
@@ -4248,7 +4352,7 @@
       </c>
     </row>
     <row r="120" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A120" s="4" t="n">
+      <c r="A120" s="5" t="n">
         <v>29526</v>
       </c>
       <c r="B120" s="1" t="n">
@@ -4281,7 +4385,7 @@
       </c>
     </row>
     <row r="121" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A121" s="4" t="n">
+      <c r="A121" s="5" t="n">
         <v>29556</v>
       </c>
       <c r="B121" s="1" t="n">
@@ -4314,7 +4418,7 @@
       </c>
     </row>
     <row r="122" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A122" s="4" t="n">
+      <c r="A122" s="5" t="n">
         <v>29587</v>
       </c>
       <c r="B122" s="1" t="n">
@@ -4347,7 +4451,7 @@
       </c>
     </row>
     <row r="123" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A123" s="4" t="n">
+      <c r="A123" s="5" t="n">
         <v>29618</v>
       </c>
       <c r="B123" s="1" t="n">
@@ -4380,7 +4484,7 @@
       </c>
     </row>
     <row r="124" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="4" t="n">
+      <c r="A124" s="5" t="n">
         <v>29646</v>
       </c>
       <c r="B124" s="1" t="n">
@@ -4413,7 +4517,7 @@
       </c>
     </row>
     <row r="125" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A125" s="4" t="n">
+      <c r="A125" s="5" t="n">
         <v>29677</v>
       </c>
       <c r="B125" s="1" t="n">
@@ -4446,7 +4550,7 @@
       </c>
     </row>
     <row r="126" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A126" s="4" t="n">
+      <c r="A126" s="5" t="n">
         <v>29707</v>
       </c>
       <c r="B126" s="1" t="n">
@@ -4479,7 +4583,7 @@
       </c>
     </row>
     <row r="127" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A127" s="4" t="n">
+      <c r="A127" s="5" t="n">
         <v>29738</v>
       </c>
       <c r="B127" s="1" t="n">
@@ -4512,7 +4616,7 @@
       </c>
     </row>
     <row r="128" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A128" s="4" t="n">
+      <c r="A128" s="5" t="n">
         <v>29768</v>
       </c>
       <c r="B128" s="1" t="n">
@@ -4545,7 +4649,7 @@
       </c>
     </row>
     <row r="129" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A129" s="4" t="n">
+      <c r="A129" s="5" t="n">
         <v>29799</v>
       </c>
       <c r="B129" s="1" t="n">
@@ -4578,7 +4682,7 @@
       </c>
     </row>
     <row r="130" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A130" s="4" t="n">
+      <c r="A130" s="5" t="n">
         <v>29830</v>
       </c>
       <c r="B130" s="1" t="n">
@@ -4611,7 +4715,7 @@
       </c>
     </row>
     <row r="131" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A131" s="4" t="n">
+      <c r="A131" s="5" t="n">
         <v>29860</v>
       </c>
       <c r="B131" s="1" t="n">
@@ -4644,7 +4748,7 @@
       </c>
     </row>
     <row r="132" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A132" s="4" t="n">
+      <c r="A132" s="5" t="n">
         <v>29891</v>
       </c>
       <c r="B132" s="1" t="n">
@@ -4677,7 +4781,7 @@
       </c>
     </row>
     <row r="133" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A133" s="4" t="n">
+      <c r="A133" s="5" t="n">
         <v>29921</v>
       </c>
       <c r="B133" s="1" t="n">
@@ -4710,7 +4814,7 @@
       </c>
     </row>
     <row r="134" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A134" s="4" t="n">
+      <c r="A134" s="5" t="n">
         <v>29952</v>
       </c>
       <c r="B134" s="1" t="n">
@@ -4743,7 +4847,7 @@
       </c>
     </row>
     <row r="135" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A135" s="4" t="n">
+      <c r="A135" s="5" t="n">
         <v>29983</v>
       </c>
       <c r="B135" s="1" t="n">
@@ -4776,7 +4880,7 @@
       </c>
     </row>
     <row r="136" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="4" t="n">
+      <c r="A136" s="5" t="n">
         <v>30011</v>
       </c>
       <c r="B136" s="1" t="n">
@@ -4809,7 +4913,7 @@
       </c>
     </row>
     <row r="137" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="4" t="n">
+      <c r="A137" s="5" t="n">
         <v>30042</v>
       </c>
       <c r="B137" s="1" t="n">
@@ -4842,7 +4946,7 @@
       </c>
     </row>
     <row r="138" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="4" t="n">
+      <c r="A138" s="5" t="n">
         <v>30072</v>
       </c>
       <c r="B138" s="1" t="n">
@@ -4875,7 +4979,7 @@
       </c>
     </row>
     <row r="139" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="4" t="n">
+      <c r="A139" s="5" t="n">
         <v>30103</v>
       </c>
       <c r="B139" s="1" t="n">
@@ -4908,7 +5012,7 @@
       </c>
     </row>
     <row r="140" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A140" s="4" t="n">
+      <c r="A140" s="5" t="n">
         <v>30133</v>
       </c>
       <c r="B140" s="1" t="n">
@@ -4941,7 +5045,7 @@
       </c>
     </row>
     <row r="141" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="4" t="n">
+      <c r="A141" s="5" t="n">
         <v>30164</v>
       </c>
       <c r="B141" s="1" t="n">
@@ -4974,7 +5078,7 @@
       </c>
     </row>
     <row r="142" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="4" t="n">
+      <c r="A142" s="5" t="n">
         <v>30195</v>
       </c>
       <c r="B142" s="1" t="n">
@@ -5007,7 +5111,7 @@
       </c>
     </row>
     <row r="143" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A143" s="4" t="n">
+      <c r="A143" s="5" t="n">
         <v>30225</v>
       </c>
       <c r="B143" s="1" t="n">
@@ -5040,7 +5144,7 @@
       </c>
     </row>
     <row r="144" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="4" t="n">
+      <c r="A144" s="5" t="n">
         <v>30256</v>
       </c>
       <c r="B144" s="1" t="n">
@@ -5073,7 +5177,7 @@
       </c>
     </row>
     <row r="145" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="4" t="n">
+      <c r="A145" s="5" t="n">
         <v>30286</v>
       </c>
       <c r="B145" s="1" t="n">
@@ -5106,7 +5210,7 @@
       </c>
     </row>
     <row r="146" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="4" t="n">
+      <c r="A146" s="5" t="n">
         <v>30317</v>
       </c>
       <c r="B146" s="1" t="n">
@@ -5139,7 +5243,7 @@
       </c>
     </row>
     <row r="147" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A147" s="4" t="n">
+      <c r="A147" s="5" t="n">
         <v>30348</v>
       </c>
       <c r="B147" s="1" t="n">
@@ -5172,7 +5276,7 @@
       </c>
     </row>
     <row r="148" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A148" s="4" t="n">
+      <c r="A148" s="5" t="n">
         <v>30376</v>
       </c>
       <c r="B148" s="1" t="n">
@@ -5205,7 +5309,7 @@
       </c>
     </row>
     <row r="149" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A149" s="4" t="n">
+      <c r="A149" s="5" t="n">
         <v>30407</v>
       </c>
       <c r="B149" s="1" t="n">
@@ -5238,7 +5342,7 @@
       </c>
     </row>
     <row r="150" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A150" s="4" t="n">
+      <c r="A150" s="5" t="n">
         <v>30437</v>
       </c>
       <c r="B150" s="1" t="n">
@@ -5271,7 +5375,7 @@
       </c>
     </row>
     <row r="151" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A151" s="4" t="n">
+      <c r="A151" s="5" t="n">
         <v>30468</v>
       </c>
       <c r="B151" s="1" t="n">
@@ -5304,7 +5408,7 @@
       </c>
     </row>
     <row r="152" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A152" s="4" t="n">
+      <c r="A152" s="5" t="n">
         <v>30498</v>
       </c>
       <c r="B152" s="1" t="n">
@@ -5337,7 +5441,7 @@
       </c>
     </row>
     <row r="153" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A153" s="4" t="n">
+      <c r="A153" s="5" t="n">
         <v>30529</v>
       </c>
       <c r="B153" s="1" t="n">
@@ -5370,7 +5474,7 @@
       </c>
     </row>
     <row r="154" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A154" s="4" t="n">
+      <c r="A154" s="5" t="n">
         <v>30560</v>
       </c>
       <c r="B154" s="1" t="n">
@@ -5403,7 +5507,7 @@
       </c>
     </row>
     <row r="155" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="4" t="n">
+      <c r="A155" s="5" t="n">
         <v>30590</v>
       </c>
       <c r="B155" s="1" t="n">
@@ -5436,7 +5540,7 @@
       </c>
     </row>
     <row r="156" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A156" s="4" t="n">
+      <c r="A156" s="5" t="n">
         <v>30621</v>
       </c>
       <c r="B156" s="1" t="n">
@@ -5469,7 +5573,7 @@
       </c>
     </row>
     <row r="157" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A157" s="4" t="n">
+      <c r="A157" s="5" t="n">
         <v>30651</v>
       </c>
       <c r="B157" s="1" t="n">
@@ -5502,7 +5606,7 @@
       </c>
     </row>
     <row r="158" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A158" s="4" t="n">
+      <c r="A158" s="5" t="n">
         <v>30682</v>
       </c>
       <c r="B158" s="1" t="n">
@@ -5535,7 +5639,7 @@
       </c>
     </row>
     <row r="159" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A159" s="4" t="n">
+      <c r="A159" s="5" t="n">
         <v>30713</v>
       </c>
       <c r="B159" s="1" t="n">
@@ -5568,7 +5672,7 @@
       </c>
     </row>
     <row r="160" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="4" t="n">
+      <c r="A160" s="5" t="n">
         <v>30742</v>
       </c>
       <c r="B160" s="1" t="n">
@@ -5601,7 +5705,7 @@
       </c>
     </row>
     <row r="161" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A161" s="4" t="n">
+      <c r="A161" s="5" t="n">
         <v>30773</v>
       </c>
       <c r="B161" s="1" t="n">
@@ -5634,7 +5738,7 @@
       </c>
     </row>
     <row r="162" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A162" s="4" t="n">
+      <c r="A162" s="5" t="n">
         <v>30803</v>
       </c>
       <c r="B162" s="1" t="n">
@@ -5667,7 +5771,7 @@
       </c>
     </row>
     <row r="163" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A163" s="4" t="n">
+      <c r="A163" s="5" t="n">
         <v>30834</v>
       </c>
       <c r="B163" s="1" t="n">
@@ -5700,7 +5804,7 @@
       </c>
     </row>
     <row r="164" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A164" s="4" t="n">
+      <c r="A164" s="5" t="n">
         <v>30864</v>
       </c>
       <c r="B164" s="1" t="n">
@@ -5733,7 +5837,7 @@
       </c>
     </row>
     <row r="165" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A165" s="4" t="n">
+      <c r="A165" s="5" t="n">
         <v>30895</v>
       </c>
       <c r="B165" s="1" t="n">
@@ -5766,7 +5870,7 @@
       </c>
     </row>
     <row r="166" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A166" s="4" t="n">
+      <c r="A166" s="5" t="n">
         <v>30926</v>
       </c>
       <c r="B166" s="1" t="n">
@@ -5799,7 +5903,7 @@
       </c>
     </row>
     <row r="167" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A167" s="4" t="n">
+      <c r="A167" s="5" t="n">
         <v>30956</v>
       </c>
       <c r="B167" s="1" t="n">
@@ -5832,7 +5936,7 @@
       </c>
     </row>
     <row r="168" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="4" t="n">
+      <c r="A168" s="5" t="n">
         <v>30987</v>
       </c>
       <c r="B168" s="1" t="n">
@@ -5865,7 +5969,7 @@
       </c>
     </row>
     <row r="169" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A169" s="4" t="n">
+      <c r="A169" s="5" t="n">
         <v>31017</v>
       </c>
       <c r="B169" s="1" t="n">
@@ -5898,7 +6002,7 @@
       </c>
     </row>
     <row r="170" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A170" s="4" t="n">
+      <c r="A170" s="5" t="n">
         <v>31048</v>
       </c>
       <c r="B170" s="1" t="n">
@@ -5931,7 +6035,7 @@
       </c>
     </row>
     <row r="171" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A171" s="4" t="n">
+      <c r="A171" s="5" t="n">
         <v>31079</v>
       </c>
       <c r="B171" s="1" t="n">
@@ -5964,7 +6068,7 @@
       </c>
     </row>
     <row r="172" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A172" s="4" t="n">
+      <c r="A172" s="5" t="n">
         <v>31107</v>
       </c>
       <c r="B172" s="1" t="n">
@@ -5997,7 +6101,7 @@
       </c>
     </row>
     <row r="173" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A173" s="4" t="n">
+      <c r="A173" s="5" t="n">
         <v>31138</v>
       </c>
       <c r="B173" s="1" t="n">
@@ -6030,7 +6134,7 @@
       </c>
     </row>
     <row r="174" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A174" s="4" t="n">
+      <c r="A174" s="5" t="n">
         <v>31168</v>
       </c>
       <c r="B174" s="1" t="n">
@@ -6063,7 +6167,7 @@
       </c>
     </row>
     <row r="175" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A175" s="4" t="n">
+      <c r="A175" s="5" t="n">
         <v>31199</v>
       </c>
       <c r="B175" s="1" t="n">
@@ -6096,7 +6200,7 @@
       </c>
     </row>
     <row r="176" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A176" s="4" t="n">
+      <c r="A176" s="5" t="n">
         <v>31229</v>
       </c>
       <c r="B176" s="1" t="n">
@@ -6129,7 +6233,7 @@
       </c>
     </row>
     <row r="177" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A177" s="4" t="n">
+      <c r="A177" s="5" t="n">
         <v>31260</v>
       </c>
       <c r="B177" s="1" t="n">
@@ -6162,7 +6266,7 @@
       </c>
     </row>
     <row r="178" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A178" s="4" t="n">
+      <c r="A178" s="5" t="n">
         <v>31291</v>
       </c>
       <c r="B178" s="1" t="n">
@@ -6195,7 +6299,7 @@
       </c>
     </row>
     <row r="179" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A179" s="4" t="n">
+      <c r="A179" s="5" t="n">
         <v>31321</v>
       </c>
       <c r="B179" s="1" t="n">
@@ -6228,7 +6332,7 @@
       </c>
     </row>
     <row r="180" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A180" s="4" t="n">
+      <c r="A180" s="5" t="n">
         <v>31352</v>
       </c>
       <c r="B180" s="1" t="n">
@@ -6261,7 +6365,7 @@
       </c>
     </row>
     <row r="181" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A181" s="4" t="n">
+      <c r="A181" s="5" t="n">
         <v>31382</v>
       </c>
       <c r="B181" s="1" t="n">
@@ -6294,7 +6398,7 @@
       </c>
     </row>
     <row r="182" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A182" s="4" t="n">
+      <c r="A182" s="5" t="n">
         <v>31413</v>
       </c>
       <c r="B182" s="1" t="n">
@@ -6327,7 +6431,7 @@
       </c>
     </row>
     <row r="183" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A183" s="4" t="n">
+      <c r="A183" s="5" t="n">
         <v>31444</v>
       </c>
       <c r="B183" s="1" t="n">
@@ -6360,7 +6464,7 @@
       </c>
     </row>
     <row r="184" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A184" s="4" t="n">
+      <c r="A184" s="5" t="n">
         <v>31472</v>
       </c>
       <c r="B184" s="1" t="n">
@@ -6393,7 +6497,7 @@
       </c>
     </row>
     <row r="185" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A185" s="4" t="n">
+      <c r="A185" s="5" t="n">
         <v>31503</v>
       </c>
       <c r="B185" s="1" t="n">
@@ -6426,7 +6530,7 @@
       </c>
     </row>
     <row r="186" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A186" s="4" t="n">
+      <c r="A186" s="5" t="n">
         <v>31533</v>
       </c>
       <c r="B186" s="1" t="n">
@@ -6459,7 +6563,7 @@
       </c>
     </row>
     <row r="187" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A187" s="4" t="n">
+      <c r="A187" s="5" t="n">
         <v>31564</v>
       </c>
       <c r="B187" s="1" t="n">
@@ -6492,7 +6596,7 @@
       </c>
     </row>
     <row r="188" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A188" s="4" t="n">
+      <c r="A188" s="5" t="n">
         <v>31594</v>
       </c>
       <c r="B188" s="1" t="n">
@@ -6525,7 +6629,7 @@
       </c>
     </row>
     <row r="189" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A189" s="4" t="n">
+      <c r="A189" s="5" t="n">
         <v>31625</v>
       </c>
       <c r="B189" s="1" t="n">
@@ -6558,7 +6662,7 @@
       </c>
     </row>
     <row r="190" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A190" s="4" t="n">
+      <c r="A190" s="5" t="n">
         <v>31656</v>
       </c>
       <c r="B190" s="1" t="n">
@@ -6591,7 +6695,7 @@
       </c>
     </row>
     <row r="191" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A191" s="4" t="n">
+      <c r="A191" s="5" t="n">
         <v>31686</v>
       </c>
       <c r="B191" s="1" t="n">
@@ -6624,7 +6728,7 @@
       </c>
     </row>
     <row r="192" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A192" s="4" t="n">
+      <c r="A192" s="5" t="n">
         <v>31717</v>
       </c>
       <c r="B192" s="1" t="n">
@@ -6657,7 +6761,7 @@
       </c>
     </row>
     <row r="193" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A193" s="4" t="n">
+      <c r="A193" s="5" t="n">
         <v>31747</v>
       </c>
       <c r="B193" s="1" t="n">
@@ -6690,7 +6794,7 @@
       </c>
     </row>
     <row r="194" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A194" s="4" t="n">
+      <c r="A194" s="5" t="n">
         <v>31778</v>
       </c>
       <c r="B194" s="1" t="n">
@@ -6723,7 +6827,7 @@
       </c>
     </row>
     <row r="195" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A195" s="4" t="n">
+      <c r="A195" s="5" t="n">
         <v>31809</v>
       </c>
       <c r="B195" s="1" t="n">
@@ -6756,7 +6860,7 @@
       </c>
     </row>
     <row r="196" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A196" s="4" t="n">
+      <c r="A196" s="5" t="n">
         <v>31837</v>
       </c>
       <c r="B196" s="1" t="n">
@@ -6789,7 +6893,7 @@
       </c>
     </row>
     <row r="197" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A197" s="4" t="n">
+      <c r="A197" s="5" t="n">
         <v>31868</v>
       </c>
       <c r="B197" s="1" t="n">
@@ -6822,7 +6926,7 @@
       </c>
     </row>
     <row r="198" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A198" s="4" t="n">
+      <c r="A198" s="5" t="n">
         <v>31898</v>
       </c>
       <c r="B198" s="1" t="n">
@@ -6855,7 +6959,7 @@
       </c>
     </row>
     <row r="199" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A199" s="4" t="n">
+      <c r="A199" s="5" t="n">
         <v>31929</v>
       </c>
       <c r="B199" s="1" t="n">
@@ -6888,7 +6992,7 @@
       </c>
     </row>
     <row r="200" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A200" s="4" t="n">
+      <c r="A200" s="5" t="n">
         <v>31959</v>
       </c>
       <c r="B200" s="1" t="n">
@@ -6921,7 +7025,7 @@
       </c>
     </row>
     <row r="201" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A201" s="4" t="n">
+      <c r="A201" s="5" t="n">
         <v>31990</v>
       </c>
       <c r="B201" s="1" t="n">
@@ -6954,7 +7058,7 @@
       </c>
     </row>
     <row r="202" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A202" s="4" t="n">
+      <c r="A202" s="5" t="n">
         <v>32021</v>
       </c>
       <c r="B202" s="1" t="n">
@@ -6987,7 +7091,7 @@
       </c>
     </row>
     <row r="203" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A203" s="4" t="n">
+      <c r="A203" s="5" t="n">
         <v>32051</v>
       </c>
       <c r="B203" s="1" t="n">
@@ -7020,7 +7124,7 @@
       </c>
     </row>
     <row r="204" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A204" s="4" t="n">
+      <c r="A204" s="5" t="n">
         <v>32082</v>
       </c>
       <c r="B204" s="1" t="n">
@@ -7053,7 +7157,7 @@
       </c>
     </row>
     <row r="205" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A205" s="4" t="n">
+      <c r="A205" s="5" t="n">
         <v>32112</v>
       </c>
       <c r="B205" s="1" t="n">
@@ -7086,7 +7190,7 @@
       </c>
     </row>
     <row r="206" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A206" s="4" t="n">
+      <c r="A206" s="5" t="n">
         <v>32143</v>
       </c>
       <c r="B206" s="1" t="n">
@@ -7119,7 +7223,7 @@
       </c>
     </row>
     <row r="207" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A207" s="4" t="n">
+      <c r="A207" s="5" t="n">
         <v>32174</v>
       </c>
       <c r="B207" s="1" t="n">
@@ -7152,7 +7256,7 @@
       </c>
     </row>
     <row r="208" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A208" s="4" t="n">
+      <c r="A208" s="5" t="n">
         <v>32203</v>
       </c>
       <c r="B208" s="1" t="n">
@@ -7185,7 +7289,7 @@
       </c>
     </row>
     <row r="209" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A209" s="4" t="n">
+      <c r="A209" s="5" t="n">
         <v>32234</v>
       </c>
       <c r="B209" s="1" t="n">
@@ -7218,7 +7322,7 @@
       </c>
     </row>
     <row r="210" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A210" s="4" t="n">
+      <c r="A210" s="5" t="n">
         <v>32264</v>
       </c>
       <c r="B210" s="1" t="n">
@@ -7251,7 +7355,7 @@
       </c>
     </row>
     <row r="211" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A211" s="4" t="n">
+      <c r="A211" s="5" t="n">
         <v>32295</v>
       </c>
       <c r="B211" s="1" t="n">
@@ -7284,7 +7388,7 @@
       </c>
     </row>
     <row r="212" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A212" s="4" t="n">
+      <c r="A212" s="5" t="n">
         <v>32325</v>
       </c>
       <c r="B212" s="1" t="n">
@@ -7317,7 +7421,7 @@
       </c>
     </row>
     <row r="213" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A213" s="4" t="n">
+      <c r="A213" s="5" t="n">
         <v>32356</v>
       </c>
       <c r="B213" s="1" t="n">
@@ -7350,7 +7454,7 @@
       </c>
     </row>
     <row r="214" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A214" s="4" t="n">
+      <c r="A214" s="5" t="n">
         <v>32387</v>
       </c>
       <c r="B214" s="1" t="n">
@@ -7383,7 +7487,7 @@
       </c>
     </row>
     <row r="215" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A215" s="4" t="n">
+      <c r="A215" s="5" t="n">
         <v>32417</v>
       </c>
       <c r="B215" s="1" t="n">
@@ -7416,7 +7520,7 @@
       </c>
     </row>
     <row r="216" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A216" s="4" t="n">
+      <c r="A216" s="5" t="n">
         <v>32448</v>
       </c>
       <c r="B216" s="1" t="n">
@@ -7449,7 +7553,7 @@
       </c>
     </row>
     <row r="217" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A217" s="4" t="n">
+      <c r="A217" s="5" t="n">
         <v>32478</v>
       </c>
       <c r="B217" s="1" t="n">
@@ -7482,7 +7586,7 @@
       </c>
     </row>
     <row r="218" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A218" s="4" t="n">
+      <c r="A218" s="5" t="n">
         <v>32509</v>
       </c>
       <c r="B218" s="1" t="n">
@@ -7515,7 +7619,7 @@
       </c>
     </row>
     <row r="219" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A219" s="4" t="n">
+      <c r="A219" s="5" t="n">
         <v>32540</v>
       </c>
       <c r="B219" s="1" t="n">
@@ -7548,7 +7652,7 @@
       </c>
     </row>
     <row r="220" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A220" s="4" t="n">
+      <c r="A220" s="5" t="n">
         <v>32568</v>
       </c>
       <c r="B220" s="1" t="n">
@@ -7581,7 +7685,7 @@
       </c>
     </row>
     <row r="221" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A221" s="4" t="n">
+      <c r="A221" s="5" t="n">
         <v>32599</v>
       </c>
       <c r="B221" s="1" t="n">
@@ -7614,7 +7718,7 @@
       </c>
     </row>
     <row r="222" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A222" s="4" t="n">
+      <c r="A222" s="5" t="n">
         <v>32629</v>
       </c>
       <c r="B222" s="1" t="n">
@@ -7647,7 +7751,7 @@
       </c>
     </row>
     <row r="223" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A223" s="4" t="n">
+      <c r="A223" s="5" t="n">
         <v>32660</v>
       </c>
       <c r="B223" s="1" t="n">
@@ -7680,7 +7784,7 @@
       </c>
     </row>
     <row r="224" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A224" s="4" t="n">
+      <c r="A224" s="5" t="n">
         <v>32690</v>
       </c>
       <c r="B224" s="1" t="n">
@@ -7713,7 +7817,7 @@
       </c>
     </row>
     <row r="225" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A225" s="4" t="n">
+      <c r="A225" s="5" t="n">
         <v>32721</v>
       </c>
       <c r="B225" s="1" t="n">
@@ -7746,7 +7850,7 @@
       </c>
     </row>
     <row r="226" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A226" s="4" t="n">
+      <c r="A226" s="5" t="n">
         <v>32752</v>
       </c>
       <c r="B226" s="1" t="n">
@@ -7779,7 +7883,7 @@
       </c>
     </row>
     <row r="227" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A227" s="4" t="n">
+      <c r="A227" s="5" t="n">
         <v>32782</v>
       </c>
       <c r="B227" s="1" t="n">
@@ -7812,7 +7916,7 @@
       </c>
     </row>
     <row r="228" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A228" s="4" t="n">
+      <c r="A228" s="5" t="n">
         <v>32813</v>
       </c>
       <c r="B228" s="1" t="n">
@@ -7845,7 +7949,7 @@
       </c>
     </row>
     <row r="229" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A229" s="4" t="n">
+      <c r="A229" s="5" t="n">
         <v>32843</v>
       </c>
       <c r="B229" s="1" t="n">
@@ -7878,7 +7982,7 @@
       </c>
     </row>
     <row r="230" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A230" s="4" t="n">
+      <c r="A230" s="5" t="n">
         <v>32874</v>
       </c>
       <c r="B230" s="1" t="n">
@@ -7911,7 +8015,7 @@
       </c>
     </row>
     <row r="231" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A231" s="4" t="n">
+      <c r="A231" s="5" t="n">
         <v>32905</v>
       </c>
       <c r="B231" s="1" t="n">
@@ -7944,7 +8048,7 @@
       </c>
     </row>
     <row r="232" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A232" s="4" t="n">
+      <c r="A232" s="5" t="n">
         <v>32933</v>
       </c>
       <c r="B232" s="1" t="n">
@@ -7977,7 +8081,7 @@
       </c>
     </row>
     <row r="233" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A233" s="4" t="n">
+      <c r="A233" s="5" t="n">
         <v>32964</v>
       </c>
       <c r="B233" s="1" t="n">
@@ -8010,7 +8114,7 @@
       </c>
     </row>
     <row r="234" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A234" s="4" t="n">
+      <c r="A234" s="5" t="n">
         <v>32994</v>
       </c>
       <c r="B234" s="1" t="n">
@@ -8043,7 +8147,7 @@
       </c>
     </row>
     <row r="235" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A235" s="4" t="n">
+      <c r="A235" s="5" t="n">
         <v>33025</v>
       </c>
       <c r="B235" s="1" t="n">
@@ -8076,7 +8180,7 @@
       </c>
     </row>
     <row r="236" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A236" s="4" t="n">
+      <c r="A236" s="5" t="n">
         <v>33055</v>
       </c>
       <c r="B236" s="1" t="n">
@@ -8109,7 +8213,7 @@
       </c>
     </row>
     <row r="237" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A237" s="4" t="n">
+      <c r="A237" s="5" t="n">
         <v>33086</v>
       </c>
       <c r="B237" s="1" t="n">
@@ -8142,7 +8246,7 @@
       </c>
     </row>
     <row r="238" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A238" s="4" t="n">
+      <c r="A238" s="5" t="n">
         <v>33117</v>
       </c>
       <c r="B238" s="1" t="n">
@@ -8175,7 +8279,7 @@
       </c>
     </row>
     <row r="239" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A239" s="4" t="n">
+      <c r="A239" s="5" t="n">
         <v>33147</v>
       </c>
       <c r="B239" s="1" t="n">
@@ -8208,7 +8312,7 @@
       </c>
     </row>
     <row r="240" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A240" s="4" t="n">
+      <c r="A240" s="5" t="n">
         <v>33178</v>
       </c>
       <c r="B240" s="1" t="n">
@@ -8241,7 +8345,7 @@
       </c>
     </row>
     <row r="241" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A241" s="4" t="n">
+      <c r="A241" s="5" t="n">
         <v>33208</v>
       </c>
       <c r="B241" s="1" t="n">
@@ -8274,7 +8378,7 @@
       </c>
     </row>
     <row r="242" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A242" s="4" t="n">
+      <c r="A242" s="5" t="n">
         <v>33239</v>
       </c>
       <c r="B242" s="1" t="n">
@@ -8307,7 +8411,7 @@
       </c>
     </row>
     <row r="243" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A243" s="4" t="n">
+      <c r="A243" s="5" t="n">
         <v>33270</v>
       </c>
       <c r="B243" s="1" t="n">
@@ -8340,7 +8444,7 @@
       </c>
     </row>
     <row r="244" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A244" s="4" t="n">
+      <c r="A244" s="5" t="n">
         <v>33298</v>
       </c>
       <c r="B244" s="1" t="n">
@@ -8373,7 +8477,7 @@
       </c>
     </row>
     <row r="245" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A245" s="4" t="n">
+      <c r="A245" s="5" t="n">
         <v>33329</v>
       </c>
       <c r="B245" s="1" t="n">
@@ -8406,7 +8510,7 @@
       </c>
     </row>
     <row r="246" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A246" s="4" t="n">
+      <c r="A246" s="5" t="n">
         <v>33359</v>
       </c>
       <c r="B246" s="1" t="n">
@@ -8439,7 +8543,7 @@
       </c>
     </row>
     <row r="247" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A247" s="4" t="n">
+      <c r="A247" s="5" t="n">
         <v>33390</v>
       </c>
       <c r="B247" s="1" t="n">
@@ -8472,7 +8576,7 @@
       </c>
     </row>
     <row r="248" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A248" s="4" t="n">
+      <c r="A248" s="5" t="n">
         <v>33420</v>
       </c>
       <c r="B248" s="1" t="n">
@@ -8505,7 +8609,7 @@
       </c>
     </row>
     <row r="249" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A249" s="4" t="n">
+      <c r="A249" s="5" t="n">
         <v>33451</v>
       </c>
       <c r="B249" s="1" t="n">
@@ -8538,7 +8642,7 @@
       </c>
     </row>
     <row r="250" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A250" s="4" t="n">
+      <c r="A250" s="5" t="n">
         <v>33482</v>
       </c>
       <c r="B250" s="1" t="n">
@@ -8571,7 +8675,7 @@
       </c>
     </row>
     <row r="251" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A251" s="4" t="n">
+      <c r="A251" s="5" t="n">
         <v>33512</v>
       </c>
       <c r="B251" s="1" t="n">
@@ -8604,7 +8708,7 @@
       </c>
     </row>
     <row r="252" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A252" s="4" t="n">
+      <c r="A252" s="5" t="n">
         <v>33543</v>
       </c>
       <c r="B252" s="1" t="n">
@@ -8637,7 +8741,7 @@
       </c>
     </row>
     <row r="253" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A253" s="4" t="n">
+      <c r="A253" s="5" t="n">
         <v>33573</v>
       </c>
       <c r="B253" s="1" t="n">
@@ -8670,7 +8774,7 @@
       </c>
     </row>
     <row r="254" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A254" s="4" t="n">
+      <c r="A254" s="5" t="n">
         <v>33604</v>
       </c>
       <c r="B254" s="1" t="n">
@@ -8703,7 +8807,7 @@
       </c>
     </row>
     <row r="255" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A255" s="4" t="n">
+      <c r="A255" s="5" t="n">
         <v>33635</v>
       </c>
       <c r="B255" s="1" t="n">
@@ -8736,7 +8840,7 @@
       </c>
     </row>
     <row r="256" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A256" s="4" t="n">
+      <c r="A256" s="5" t="n">
         <v>33664</v>
       </c>
       <c r="B256" s="1" t="n">
@@ -8769,7 +8873,7 @@
       </c>
     </row>
     <row r="257" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A257" s="4" t="n">
+      <c r="A257" s="5" t="n">
         <v>33695</v>
       </c>
       <c r="B257" s="1" t="n">
@@ -8802,7 +8906,7 @@
       </c>
     </row>
     <row r="258" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A258" s="4" t="n">
+      <c r="A258" s="5" t="n">
         <v>33725</v>
       </c>
       <c r="B258" s="1" t="n">
@@ -8835,7 +8939,7 @@
       </c>
     </row>
     <row r="259" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A259" s="4" t="n">
+      <c r="A259" s="5" t="n">
         <v>33756</v>
       </c>
       <c r="B259" s="1" t="n">
@@ -8868,7 +8972,7 @@
       </c>
     </row>
     <row r="260" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A260" s="4" t="n">
+      <c r="A260" s="5" t="n">
         <v>33786</v>
       </c>
       <c r="B260" s="1" t="n">
@@ -8901,7 +9005,7 @@
       </c>
     </row>
     <row r="261" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A261" s="4" t="n">
+      <c r="A261" s="5" t="n">
         <v>33817</v>
       </c>
       <c r="B261" s="1" t="n">
@@ -8934,7 +9038,7 @@
       </c>
     </row>
     <row r="262" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A262" s="4" t="n">
+      <c r="A262" s="5" t="n">
         <v>33848</v>
       </c>
       <c r="B262" s="1" t="n">
@@ -8967,7 +9071,7 @@
       </c>
     </row>
     <row r="263" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A263" s="4" t="n">
+      <c r="A263" s="5" t="n">
         <v>33878</v>
       </c>
       <c r="B263" s="1" t="n">
@@ -9000,7 +9104,7 @@
       </c>
     </row>
     <row r="264" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A264" s="4" t="n">
+      <c r="A264" s="5" t="n">
         <v>33909</v>
       </c>
       <c r="B264" s="1" t="n">
@@ -9033,7 +9137,7 @@
       </c>
     </row>
     <row r="265" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A265" s="4" t="n">
+      <c r="A265" s="5" t="n">
         <v>33939</v>
       </c>
       <c r="B265" s="1" t="n">
@@ -9066,7 +9170,7 @@
       </c>
     </row>
     <row r="266" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A266" s="4" t="n">
+      <c r="A266" s="5" t="n">
         <v>33970</v>
       </c>
       <c r="B266" s="1" t="n">
@@ -9099,7 +9203,7 @@
       </c>
     </row>
     <row r="267" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A267" s="4" t="n">
+      <c r="A267" s="5" t="n">
         <v>34001</v>
       </c>
       <c r="B267" s="1" t="n">
@@ -9132,7 +9236,7 @@
       </c>
     </row>
     <row r="268" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A268" s="4" t="n">
+      <c r="A268" s="5" t="n">
         <v>34029</v>
       </c>
       <c r="B268" s="1" t="n">
@@ -9165,7 +9269,7 @@
       </c>
     </row>
     <row r="269" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A269" s="4" t="n">
+      <c r="A269" s="5" t="n">
         <v>34060</v>
       </c>
       <c r="B269" s="1" t="n">
@@ -9198,7 +9302,7 @@
       </c>
     </row>
     <row r="270" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A270" s="4" t="n">
+      <c r="A270" s="5" t="n">
         <v>34090</v>
       </c>
       <c r="B270" s="1" t="n">
@@ -9231,7 +9335,7 @@
       </c>
     </row>
     <row r="271" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A271" s="4" t="n">
+      <c r="A271" s="5" t="n">
         <v>34121</v>
       </c>
       <c r="B271" s="1" t="n">
@@ -9264,7 +9368,7 @@
       </c>
     </row>
     <row r="272" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A272" s="4" t="n">
+      <c r="A272" s="5" t="n">
         <v>34151</v>
       </c>
       <c r="B272" s="1" t="n">
@@ -9297,7 +9401,7 @@
       </c>
     </row>
     <row r="273" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A273" s="4" t="n">
+      <c r="A273" s="5" t="n">
         <v>34182</v>
       </c>
       <c r="B273" s="1" t="n">
@@ -9330,7 +9434,7 @@
       </c>
     </row>
     <row r="274" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A274" s="4" t="n">
+      <c r="A274" s="5" t="n">
         <v>34213</v>
       </c>
       <c r="B274" s="1" t="n">
@@ -9363,7 +9467,7 @@
       </c>
     </row>
     <row r="275" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A275" s="4" t="n">
+      <c r="A275" s="5" t="n">
         <v>34243</v>
       </c>
       <c r="B275" s="1" t="n">
@@ -9396,7 +9500,7 @@
       </c>
     </row>
     <row r="276" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A276" s="4" t="n">
+      <c r="A276" s="5" t="n">
         <v>34274</v>
       </c>
       <c r="B276" s="1" t="n">
@@ -9429,7 +9533,7 @@
       </c>
     </row>
     <row r="277" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A277" s="4" t="n">
+      <c r="A277" s="5" t="n">
         <v>34304</v>
       </c>
       <c r="B277" s="1" t="n">
@@ -9462,7 +9566,7 @@
       </c>
     </row>
     <row r="278" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A278" s="4" t="n">
+      <c r="A278" s="5" t="n">
         <v>34335</v>
       </c>
       <c r="B278" s="1" t="n">
@@ -9495,7 +9599,7 @@
       </c>
     </row>
     <row r="279" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A279" s="4" t="n">
+      <c r="A279" s="5" t="n">
         <v>34366</v>
       </c>
       <c r="B279" s="1" t="n">
@@ -9528,7 +9632,7 @@
       </c>
     </row>
     <row r="280" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A280" s="4" t="n">
+      <c r="A280" s="5" t="n">
         <v>34394</v>
       </c>
       <c r="B280" s="1" t="n">
@@ -9561,7 +9665,7 @@
       </c>
     </row>
     <row r="281" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A281" s="4" t="n">
+      <c r="A281" s="5" t="n">
         <v>34425</v>
       </c>
       <c r="B281" s="1" t="n">
@@ -9594,7 +9698,7 @@
       </c>
     </row>
     <row r="282" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A282" s="4" t="n">
+      <c r="A282" s="5" t="n">
         <v>34455</v>
       </c>
       <c r="B282" s="1" t="n">
@@ -9627,7 +9731,7 @@
       </c>
     </row>
     <row r="283" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A283" s="4" t="n">
+      <c r="A283" s="5" t="n">
         <v>34486</v>
       </c>
       <c r="B283" s="1" t="n">
@@ -9660,7 +9764,7 @@
       </c>
     </row>
     <row r="284" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A284" s="4" t="n">
+      <c r="A284" s="5" t="n">
         <v>34516</v>
       </c>
       <c r="B284" s="1" t="n">
@@ -9693,7 +9797,7 @@
       </c>
     </row>
     <row r="285" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A285" s="4" t="n">
+      <c r="A285" s="5" t="n">
         <v>34547</v>
       </c>
       <c r="B285" s="1" t="n">
@@ -9726,7 +9830,7 @@
       </c>
     </row>
     <row r="286" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A286" s="4" t="n">
+      <c r="A286" s="5" t="n">
         <v>34578</v>
       </c>
       <c r="B286" s="1" t="n">
@@ -9759,7 +9863,7 @@
       </c>
     </row>
     <row r="287" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A287" s="4" t="n">
+      <c r="A287" s="5" t="n">
         <v>34608</v>
       </c>
       <c r="B287" s="1" t="n">
@@ -9792,7 +9896,7 @@
       </c>
     </row>
     <row r="288" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A288" s="4" t="n">
+      <c r="A288" s="5" t="n">
         <v>34639</v>
       </c>
       <c r="B288" s="1" t="n">
@@ -9825,7 +9929,7 @@
       </c>
     </row>
     <row r="289" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A289" s="4" t="n">
+      <c r="A289" s="5" t="n">
         <v>34669</v>
       </c>
       <c r="B289" s="1" t="n">
@@ -9858,7 +9962,7 @@
       </c>
     </row>
     <row r="290" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A290" s="4" t="n">
+      <c r="A290" s="5" t="n">
         <v>34700</v>
       </c>
       <c r="B290" s="1" t="n">
@@ -9891,7 +9995,7 @@
       </c>
     </row>
     <row r="291" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A291" s="4" t="n">
+      <c r="A291" s="5" t="n">
         <v>34731</v>
       </c>
       <c r="B291" s="1" t="n">
@@ -9924,7 +10028,7 @@
       </c>
     </row>
     <row r="292" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A292" s="4" t="n">
+      <c r="A292" s="5" t="n">
         <v>34759</v>
       </c>
       <c r="B292" s="1" t="n">
@@ -9957,7 +10061,7 @@
       </c>
     </row>
     <row r="293" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A293" s="4" t="n">
+      <c r="A293" s="5" t="n">
         <v>34790</v>
       </c>
       <c r="B293" s="1" t="n">
@@ -9990,7 +10094,7 @@
       </c>
     </row>
     <row r="294" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A294" s="4" t="n">
+      <c r="A294" s="5" t="n">
         <v>34820</v>
       </c>
       <c r="B294" s="1" t="n">
@@ -10023,7 +10127,7 @@
       </c>
     </row>
     <row r="295" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A295" s="4" t="n">
+      <c r="A295" s="5" t="n">
         <v>34851</v>
       </c>
       <c r="B295" s="1" t="n">
@@ -10056,7 +10160,7 @@
       </c>
     </row>
     <row r="296" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A296" s="4" t="n">
+      <c r="A296" s="5" t="n">
         <v>34881</v>
       </c>
       <c r="B296" s="1" t="n">
@@ -10089,7 +10193,7 @@
       </c>
     </row>
     <row r="297" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A297" s="4" t="n">
+      <c r="A297" s="5" t="n">
         <v>34912</v>
       </c>
       <c r="B297" s="1" t="n">
@@ -10122,7 +10226,7 @@
       </c>
     </row>
     <row r="298" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A298" s="4" t="n">
+      <c r="A298" s="5" t="n">
         <v>34943</v>
       </c>
       <c r="B298" s="1" t="n">
@@ -10155,7 +10259,7 @@
       </c>
     </row>
     <row r="299" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A299" s="4" t="n">
+      <c r="A299" s="5" t="n">
         <v>34973</v>
       </c>
       <c r="B299" s="1" t="n">
@@ -10188,7 +10292,7 @@
       </c>
     </row>
     <row r="300" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A300" s="4" t="n">
+      <c r="A300" s="5" t="n">
         <v>35004</v>
       </c>
       <c r="B300" s="1" t="n">
@@ -10221,7 +10325,7 @@
       </c>
     </row>
     <row r="301" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A301" s="4" t="n">
+      <c r="A301" s="5" t="n">
         <v>35034</v>
       </c>
       <c r="B301" s="1" t="n">
@@ -10254,7 +10358,7 @@
       </c>
     </row>
     <row r="302" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A302" s="4" t="n">
+      <c r="A302" s="5" t="n">
         <v>35065</v>
       </c>
       <c r="B302" s="1" t="n">
@@ -10287,7 +10391,7 @@
       </c>
     </row>
     <row r="303" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A303" s="4" t="n">
+      <c r="A303" s="5" t="n">
         <v>35096</v>
       </c>
       <c r="B303" s="1" t="n">
@@ -10320,7 +10424,7 @@
       </c>
     </row>
     <row r="304" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A304" s="4" t="n">
+      <c r="A304" s="5" t="n">
         <v>35125</v>
       </c>
       <c r="B304" s="1" t="n">
@@ -10353,7 +10457,7 @@
       </c>
     </row>
     <row r="305" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A305" s="4" t="n">
+      <c r="A305" s="5" t="n">
         <v>35156</v>
       </c>
       <c r="B305" s="1" t="n">
@@ -10386,7 +10490,7 @@
       </c>
     </row>
     <row r="306" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A306" s="4" t="n">
+      <c r="A306" s="5" t="n">
         <v>35186</v>
       </c>
       <c r="B306" s="1" t="n">
@@ -10419,7 +10523,7 @@
       </c>
     </row>
     <row r="307" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A307" s="4" t="n">
+      <c r="A307" s="5" t="n">
         <v>35217</v>
       </c>
       <c r="B307" s="1" t="n">
@@ -10452,7 +10556,7 @@
       </c>
     </row>
     <row r="308" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A308" s="4" t="n">
+      <c r="A308" s="5" t="n">
         <v>35247</v>
       </c>
       <c r="B308" s="1" t="n">
@@ -10485,7 +10589,7 @@
       </c>
     </row>
     <row r="309" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A309" s="4" t="n">
+      <c r="A309" s="5" t="n">
         <v>35278</v>
       </c>
       <c r="B309" s="1" t="n">
@@ -10518,7 +10622,7 @@
       </c>
     </row>
     <row r="310" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A310" s="4" t="n">
+      <c r="A310" s="5" t="n">
         <v>35309</v>
       </c>
       <c r="B310" s="1" t="n">
@@ -10551,7 +10655,7 @@
       </c>
     </row>
     <row r="311" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A311" s="4" t="n">
+      <c r="A311" s="5" t="n">
         <v>35339</v>
       </c>
       <c r="B311" s="1" t="n">
@@ -10584,7 +10688,7 @@
       </c>
     </row>
     <row r="312" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A312" s="4" t="n">
+      <c r="A312" s="5" t="n">
         <v>35370</v>
       </c>
       <c r="B312" s="1" t="n">
@@ -10617,7 +10721,7 @@
       </c>
     </row>
     <row r="313" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A313" s="4" t="n">
+      <c r="A313" s="5" t="n">
         <v>35400</v>
       </c>
       <c r="B313" s="1" t="n">
@@ -10650,7 +10754,7 @@
       </c>
     </row>
     <row r="314" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A314" s="4" t="n">
+      <c r="A314" s="5" t="n">
         <v>35431</v>
       </c>
       <c r="B314" s="1" t="n">
@@ -10683,7 +10787,7 @@
       </c>
     </row>
     <row r="315" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A315" s="4" t="n">
+      <c r="A315" s="5" t="n">
         <v>35462</v>
       </c>
       <c r="B315" s="1" t="n">
@@ -10716,7 +10820,7 @@
       </c>
     </row>
     <row r="316" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A316" s="4" t="n">
+      <c r="A316" s="5" t="n">
         <v>35490</v>
       </c>
       <c r="B316" s="1" t="n">
@@ -10749,7 +10853,7 @@
       </c>
     </row>
     <row r="317" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A317" s="4" t="n">
+      <c r="A317" s="5" t="n">
         <v>35521</v>
       </c>
       <c r="B317" s="1" t="n">
@@ -10782,7 +10886,7 @@
       </c>
     </row>
     <row r="318" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A318" s="4" t="n">
+      <c r="A318" s="5" t="n">
         <v>35551</v>
       </c>
       <c r="B318" s="1" t="n">
@@ -10815,7 +10919,7 @@
       </c>
     </row>
     <row r="319" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A319" s="4" t="n">
+      <c r="A319" s="5" t="n">
         <v>35582</v>
       </c>
       <c r="B319" s="1" t="n">
@@ -10848,7 +10952,7 @@
       </c>
     </row>
     <row r="320" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A320" s="4" t="n">
+      <c r="A320" s="5" t="n">
         <v>35612</v>
       </c>
       <c r="B320" s="1" t="n">
@@ -10881,7 +10985,7 @@
       </c>
     </row>
     <row r="321" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A321" s="4" t="n">
+      <c r="A321" s="5" t="n">
         <v>35643</v>
       </c>
       <c r="B321" s="1" t="n">
@@ -10914,7 +11018,7 @@
       </c>
     </row>
     <row r="322" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A322" s="4" t="n">
+      <c r="A322" s="5" t="n">
         <v>35674</v>
       </c>
       <c r="B322" s="1" t="n">
@@ -10947,7 +11051,7 @@
       </c>
     </row>
     <row r="323" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A323" s="4" t="n">
+      <c r="A323" s="5" t="n">
         <v>35704</v>
       </c>
       <c r="B323" s="1" t="n">
@@ -10980,7 +11084,7 @@
       </c>
     </row>
     <row r="324" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A324" s="4" t="n">
+      <c r="A324" s="5" t="n">
         <v>35735</v>
       </c>
       <c r="B324" s="1" t="n">
@@ -11013,7 +11117,7 @@
       </c>
     </row>
     <row r="325" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A325" s="4" t="n">
+      <c r="A325" s="5" t="n">
         <v>35765</v>
       </c>
       <c r="B325" s="1" t="n">
@@ -11046,7 +11150,7 @@
       </c>
     </row>
     <row r="326" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A326" s="4" t="n">
+      <c r="A326" s="5" t="n">
         <v>35796</v>
       </c>
       <c r="B326" s="1" t="n">
@@ -11079,7 +11183,7 @@
       </c>
     </row>
     <row r="327" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A327" s="4" t="n">
+      <c r="A327" s="5" t="n">
         <v>35827</v>
       </c>
       <c r="B327" s="1" t="n">
@@ -11112,7 +11216,7 @@
       </c>
     </row>
     <row r="328" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A328" s="4" t="n">
+      <c r="A328" s="5" t="n">
         <v>35855</v>
       </c>
       <c r="B328" s="1" t="n">
@@ -11145,7 +11249,7 @@
       </c>
     </row>
     <row r="329" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A329" s="4" t="n">
+      <c r="A329" s="5" t="n">
         <v>35886</v>
       </c>
       <c r="B329" s="1" t="n">
@@ -11178,7 +11282,7 @@
       </c>
     </row>
     <row r="330" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A330" s="4" t="n">
+      <c r="A330" s="5" t="n">
         <v>35916</v>
       </c>
       <c r="B330" s="1" t="n">
@@ -11211,7 +11315,7 @@
       </c>
     </row>
     <row r="331" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A331" s="4" t="n">
+      <c r="A331" s="5" t="n">
         <v>35947</v>
       </c>
       <c r="B331" s="1" t="n">
@@ -11244,7 +11348,7 @@
       </c>
     </row>
     <row r="332" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A332" s="4" t="n">
+      <c r="A332" s="5" t="n">
         <v>35977</v>
       </c>
       <c r="B332" s="1" t="n">
@@ -11277,7 +11381,7 @@
       </c>
     </row>
     <row r="333" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A333" s="4" t="n">
+      <c r="A333" s="5" t="n">
         <v>36008</v>
       </c>
       <c r="B333" s="1" t="n">
@@ -11310,7 +11414,7 @@
       </c>
     </row>
     <row r="334" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A334" s="4" t="n">
+      <c r="A334" s="5" t="n">
         <v>36039</v>
       </c>
       <c r="B334" s="1" t="n">
@@ -11343,7 +11447,7 @@
       </c>
     </row>
     <row r="335" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A335" s="4" t="n">
+      <c r="A335" s="5" t="n">
         <v>36069</v>
       </c>
       <c r="B335" s="1" t="n">
@@ -11376,7 +11480,7 @@
       </c>
     </row>
     <row r="336" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A336" s="4" t="n">
+      <c r="A336" s="5" t="n">
         <v>36100</v>
       </c>
       <c r="B336" s="1" t="n">
@@ -11409,7 +11513,7 @@
       </c>
     </row>
     <row r="337" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A337" s="4" t="n">
+      <c r="A337" s="5" t="n">
         <v>36130</v>
       </c>
       <c r="B337" s="1" t="n">
@@ -11442,7 +11546,7 @@
       </c>
     </row>
     <row r="338" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A338" s="4" t="n">
+      <c r="A338" s="5" t="n">
         <v>36161</v>
       </c>
       <c r="B338" s="1" t="n">
@@ -11475,7 +11579,7 @@
       </c>
     </row>
     <row r="339" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A339" s="4" t="n">
+      <c r="A339" s="5" t="n">
         <v>36192</v>
       </c>
       <c r="B339" s="1" t="n">
@@ -11508,7 +11612,7 @@
       </c>
     </row>
     <row r="340" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A340" s="4" t="n">
+      <c r="A340" s="5" t="n">
         <v>36220</v>
       </c>
       <c r="B340" s="1" t="n">
@@ -11541,7 +11645,7 @@
       </c>
     </row>
     <row r="341" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A341" s="4" t="n">
+      <c r="A341" s="5" t="n">
         <v>36251</v>
       </c>
       <c r="B341" s="1" t="n">
@@ -11574,7 +11678,7 @@
       </c>
     </row>
     <row r="342" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A342" s="4" t="n">
+      <c r="A342" s="5" t="n">
         <v>36281</v>
       </c>
       <c r="B342" s="1" t="n">
@@ -11607,7 +11711,7 @@
       </c>
     </row>
     <row r="343" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A343" s="4" t="n">
+      <c r="A343" s="5" t="n">
         <v>36312</v>
       </c>
       <c r="B343" s="1" t="n">
@@ -11640,7 +11744,7 @@
       </c>
     </row>
     <row r="344" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A344" s="4" t="n">
+      <c r="A344" s="5" t="n">
         <v>36342</v>
       </c>
       <c r="B344" s="1" t="n">
@@ -11673,7 +11777,7 @@
       </c>
     </row>
     <row r="345" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A345" s="4" t="n">
+      <c r="A345" s="5" t="n">
         <v>36373</v>
       </c>
       <c r="B345" s="1" t="n">
@@ -11706,7 +11810,7 @@
       </c>
     </row>
     <row r="346" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A346" s="4" t="n">
+      <c r="A346" s="5" t="n">
         <v>36404</v>
       </c>
       <c r="B346" s="1" t="n">
@@ -11739,7 +11843,7 @@
       </c>
     </row>
     <row r="347" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A347" s="4" t="n">
+      <c r="A347" s="5" t="n">
         <v>36434</v>
       </c>
       <c r="B347" s="1" t="n">
@@ -11772,7 +11876,7 @@
       </c>
     </row>
     <row r="348" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A348" s="4" t="n">
+      <c r="A348" s="5" t="n">
         <v>36465</v>
       </c>
       <c r="B348" s="1" t="n">
@@ -11805,7 +11909,7 @@
       </c>
     </row>
     <row r="349" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A349" s="4" t="n">
+      <c r="A349" s="5" t="n">
         <v>36495</v>
       </c>
       <c r="B349" s="1" t="n">
@@ -11838,7 +11942,7 @@
       </c>
     </row>
     <row r="350" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A350" s="4" t="n">
+      <c r="A350" s="5" t="n">
         <v>36526</v>
       </c>
       <c r="B350" s="1" t="n">
@@ -11871,7 +11975,7 @@
       </c>
     </row>
     <row r="351" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A351" s="4" t="n">
+      <c r="A351" s="5" t="n">
         <v>36557</v>
       </c>
       <c r="B351" s="1" t="n">
@@ -11904,7 +12008,7 @@
       </c>
     </row>
     <row r="352" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A352" s="4" t="n">
+      <c r="A352" s="5" t="n">
         <v>36586</v>
       </c>
       <c r="B352" s="1" t="n">
@@ -11937,7 +12041,7 @@
       </c>
     </row>
     <row r="353" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A353" s="4" t="n">
+      <c r="A353" s="5" t="n">
         <v>36617</v>
       </c>
       <c r="B353" s="1" t="n">
@@ -11970,7 +12074,7 @@
       </c>
     </row>
     <row r="354" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A354" s="4" t="n">
+      <c r="A354" s="5" t="n">
         <v>36647</v>
       </c>
       <c r="B354" s="1" t="n">
@@ -12003,7 +12107,7 @@
       </c>
     </row>
     <row r="355" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A355" s="4" t="n">
+      <c r="A355" s="5" t="n">
         <v>36678</v>
       </c>
       <c r="B355" s="1" t="n">
@@ -12036,7 +12140,7 @@
       </c>
     </row>
     <row r="356" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A356" s="4" t="n">
+      <c r="A356" s="5" t="n">
         <v>36708</v>
       </c>
       <c r="B356" s="1" t="n">
@@ -12069,7 +12173,7 @@
       </c>
     </row>
     <row r="357" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A357" s="4" t="n">
+      <c r="A357" s="5" t="n">
         <v>36739</v>
       </c>
       <c r="B357" s="1" t="n">
@@ -12102,7 +12206,7 @@
       </c>
     </row>
     <row r="358" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A358" s="4" t="n">
+      <c r="A358" s="5" t="n">
         <v>36770</v>
       </c>
       <c r="B358" s="1" t="n">
@@ -12135,7 +12239,7 @@
       </c>
     </row>
     <row r="359" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A359" s="4" t="n">
+      <c r="A359" s="5" t="n">
         <v>36800</v>
       </c>
       <c r="B359" s="1" t="n">
@@ -12168,7 +12272,7 @@
       </c>
     </row>
     <row r="360" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A360" s="4" t="n">
+      <c r="A360" s="5" t="n">
         <v>36831</v>
       </c>
       <c r="B360" s="1" t="n">
@@ -12201,7 +12305,7 @@
       </c>
     </row>
     <row r="361" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A361" s="4" t="n">
+      <c r="A361" s="5" t="n">
         <v>36861</v>
       </c>
       <c r="B361" s="1" t="n">
@@ -12245,23 +12349,23 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="35.01"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="1" t="n">
@@ -12270,7 +12374,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="1" t="n">
@@ -12279,24 +12383,24 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="6" t="n">
+      <c r="C4" s="7" t="n">
         <f aca="false">C2/C3</f>
         <v>0.128251396522217</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="6"/>
+      <c r="B5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="1" t="n">
@@ -12305,72 +12409,73 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7" t="n">
+      <c r="C8" s="8" t="n">
         <f aca="false">STDEV(Data!K2:K361)</f>
         <v>0.0307130967387096</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="7" t="n">
         <f aca="false">C7/C8</f>
         <v>0.116589784605477</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="7" t="n">
         <f aca="false">SLOPE(Data!K2:K361,Data!G2:G361)</f>
         <v>-0.194966881553934</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="7" t="n">
+      <c r="C11" s="8" t="n">
         <f aca="false">INTERCEPT(Data!K2:K361,Data!G2:G361)</f>
         <v>0.00472978399782408</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="7" t="n">
         <f aca="false">C11 / SQRT( C8^2 - C10^2*C3^2)</f>
         <v>0.161000164109882</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <f aca="false">SQRT(C4^2 + C12^2)</f>
         <v>0.205838464707907</v>
       </c>
     </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="s">
+      <c r="A17" s="9" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C18" s="1" t="n">
@@ -12379,67 +12484,68 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="10" t="n">
         <f aca="false">PRODUCT('At 1% exc return vol'!C2:C361)</f>
         <v>10.8119316147417</v>
       </c>
     </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G23" s="0" t="s">
+      <c r="G23" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="H23" s="0" t="s">
+      <c r="H23" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="1" t="n">
         <f aca="false">C2</f>
         <v>0.00589305555555556</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="E24" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="F24" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G24" s="1" t="n">
         <f aca="false">C3^2</f>
         <v>0.00211133362852058</v>
       </c>
-      <c r="H24" s="7" t="n">
+      <c r="H24" s="8" t="n">
         <f aca="false">C3*C8*CORREL(Data!G2:G361,Data!K2:K361)</f>
         <v>-0.000411640133472609</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C25" s="0" t="s">
+      <c r="C25" s="2" t="s">
         <v>29</v>
       </c>
       <c r="D25" s="1" t="n">
         <f aca="false">C7</f>
         <v>0.00358083333333333</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="F25" s="2" t="s">
         <v>25</v>
       </c>
       <c r="G25" s="1" t="n">
@@ -12453,24 +12559,25 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C27" s="0" t="n">
+      <c r="C27" s="7" t="n">
         <f aca="false" t="array" ref="C27:C28">MMULT(MINVERSE(G24:H25),D24:D25)</f>
-        <v>3.85964738746478</v>
+        <v>3.85964738746479</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C28" s="0" t="n">
+      <c r="C28" s="7" t="n">
         <v>5.48038829158666</v>
       </c>
     </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="2" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="1" t="n">
@@ -12479,7 +12586,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C31" s="1" t="n">
@@ -12487,8 +12594,9 @@
         <v>0.586763100260794</v>
       </c>
     </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C33" s="1" t="n">
@@ -12497,7 +12605,7 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C34" s="1" t="n">
@@ -12506,19 +12614,20 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="6" t="n">
+      <c r="C35" s="7" t="n">
         <f aca="false">C33/C34</f>
         <v>0.205838464707906</v>
       </c>
-      <c r="D35" s="0" t="s">
+      <c r="D35" s="2" t="s">
         <v>37</v>
       </c>
     </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="2" t="s">
         <v>20</v>
       </c>
       <c r="C37" s="1" t="n">
@@ -12527,10 +12636,10 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="0" t="s">
+      <c r="B38" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="9" t="n">
+      <c r="C38" s="10" t="n">
         <f aca="false">PRODUCT('At 1% exc return vol'!G2:G361)</f>
         <v>14.2620292807815</v>
       </c>
@@ -12547,36 +12656,36 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G361"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="41.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="8.68"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="55.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="41.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="8.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="55.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="2" t="s">
         <v>40</v>
       </c>
     </row>

</xml_diff>